<commit_message>
Se corrigio los ceros en los decimales negativos, ahora ya no existen 0 por decimales significativos
</commit_message>
<xml_diff>
--- a/datos/datos_calidad_aire_DIARIO_IAS.xlsx
+++ b/datos/datos_calidad_aire_DIARIO_IAS.xlsx
@@ -5310,14 +5310,8 @@
       <c r="BQ15" s="2" t="inlineStr"/>
       <c r="BR15" s="2" t="inlineStr"/>
       <c r="BS15" s="2" t="inlineStr"/>
-      <c r="BT15" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BU15" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="BT15" s="2" t="inlineStr"/>
+      <c r="BU15" s="2" t="inlineStr"/>
       <c r="BV15" s="3" t="inlineStr">
         <is>
           <t>Buena</t>
@@ -5940,14 +5934,8 @@
       <c r="BS17" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="BT17" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BU17" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="BT17" s="2" t="inlineStr"/>
+      <c r="BU17" s="2" t="inlineStr"/>
       <c r="BV17" s="3" t="inlineStr">
         <is>
           <t>Buena</t>
@@ -6106,14 +6094,8 @@
       <c r="U18" s="8" t="n">
         <v>47</v>
       </c>
-      <c r="V18" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W18" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V18" s="2" t="inlineStr"/>
+      <c r="W18" s="2" t="inlineStr"/>
       <c r="X18" s="2" t="inlineStr"/>
       <c r="Y18" s="2" t="inlineStr"/>
       <c r="Z18" s="3" t="inlineStr">
@@ -6424,14 +6406,8 @@
       <c r="U19" s="8" t="n">
         <v>42</v>
       </c>
-      <c r="V19" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W19" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V19" s="2" t="inlineStr"/>
+      <c r="W19" s="2" t="inlineStr"/>
       <c r="X19" s="2" t="inlineStr"/>
       <c r="Y19" s="2" t="inlineStr"/>
       <c r="Z19" s="3" t="inlineStr">
@@ -6748,14 +6724,8 @@
       <c r="U20" s="8" t="n">
         <v>39</v>
       </c>
-      <c r="V20" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W20" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V20" s="2" t="inlineStr"/>
+      <c r="W20" s="2" t="inlineStr"/>
       <c r="X20" s="2" t="inlineStr"/>
       <c r="Y20" s="2" t="inlineStr"/>
       <c r="Z20" s="3" t="inlineStr">
@@ -7072,14 +7042,8 @@
       <c r="U21" s="8" t="n">
         <v>43</v>
       </c>
-      <c r="V21" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W21" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V21" s="2" t="inlineStr"/>
+      <c r="W21" s="2" t="inlineStr"/>
       <c r="X21" s="2" t="inlineStr"/>
       <c r="Y21" s="2" t="inlineStr"/>
       <c r="Z21" s="3" t="inlineStr">
@@ -7396,14 +7360,8 @@
       <c r="U22" s="8" t="n">
         <v>40</v>
       </c>
-      <c r="V22" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W22" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V22" s="2" t="inlineStr"/>
+      <c r="W22" s="2" t="inlineStr"/>
       <c r="X22" s="2" t="inlineStr"/>
       <c r="Y22" s="2" t="inlineStr"/>
       <c r="Z22" s="3" t="inlineStr">
@@ -7538,14 +7496,8 @@
       <c r="BO22" s="5" t="n">
         <v>0.058</v>
       </c>
-      <c r="BP22" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BQ22" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="BP22" s="2" t="inlineStr"/>
+      <c r="BQ22" s="2" t="inlineStr"/>
       <c r="BR22" s="6" t="inlineStr">
         <is>
           <t>Aceptable</t>
@@ -7714,14 +7666,8 @@
       <c r="S23" s="2" t="inlineStr"/>
       <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
-      <c r="V23" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W23" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V23" s="2" t="inlineStr"/>
+      <c r="W23" s="2" t="inlineStr"/>
       <c r="X23" s="2" t="inlineStr"/>
       <c r="Y23" s="2" t="inlineStr"/>
       <c r="Z23" s="3" t="inlineStr">
@@ -7850,14 +7796,8 @@
       <c r="BO23" s="5" t="n">
         <v>0.052</v>
       </c>
-      <c r="BP23" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BQ23" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="BP23" s="2" t="inlineStr"/>
+      <c r="BQ23" s="2" t="inlineStr"/>
       <c r="BR23" s="3" t="inlineStr">
         <is>
           <t>Buena</t>
@@ -8020,14 +7960,8 @@
       <c r="U24" s="8" t="n">
         <v>36</v>
       </c>
-      <c r="V24" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W24" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V24" s="2" t="inlineStr"/>
+      <c r="W24" s="2" t="inlineStr"/>
       <c r="X24" s="2" t="inlineStr"/>
       <c r="Y24" s="2" t="inlineStr"/>
       <c r="Z24" s="3" t="inlineStr">
@@ -8150,14 +8084,8 @@
       <c r="BO24" s="5" t="n">
         <v>0.058</v>
       </c>
-      <c r="BP24" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BQ24" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="BP24" s="2" t="inlineStr"/>
+      <c r="BQ24" s="2" t="inlineStr"/>
       <c r="BR24" s="3" t="inlineStr">
         <is>
           <t>Buena</t>
@@ -8326,14 +8254,8 @@
       <c r="U25" s="8" t="n">
         <v>36</v>
       </c>
-      <c r="V25" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W25" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V25" s="2" t="inlineStr"/>
+      <c r="W25" s="2" t="inlineStr"/>
       <c r="X25" s="2" t="inlineStr"/>
       <c r="Y25" s="2" t="inlineStr"/>
       <c r="Z25" s="2" t="inlineStr"/>
@@ -8432,14 +8354,8 @@
       <c r="BO25" s="5" t="n">
         <v>0.052</v>
       </c>
-      <c r="BP25" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BQ25" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="BP25" s="2" t="inlineStr"/>
+      <c r="BQ25" s="2" t="inlineStr"/>
       <c r="BR25" s="3" t="inlineStr">
         <is>
           <t>Buena</t>
@@ -8608,14 +8524,8 @@
       <c r="U26" s="8" t="n">
         <v>43</v>
       </c>
-      <c r="V26" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W26" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V26" s="2" t="inlineStr"/>
+      <c r="W26" s="2" t="inlineStr"/>
       <c r="X26" s="2" t="inlineStr"/>
       <c r="Y26" s="2" t="inlineStr"/>
       <c r="Z26" s="2" t="inlineStr"/>
@@ -8714,14 +8624,8 @@
       <c r="BO26" s="5" t="n">
         <v>0.054</v>
       </c>
-      <c r="BP26" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BQ26" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="BP26" s="2" t="inlineStr"/>
+      <c r="BQ26" s="2" t="inlineStr"/>
       <c r="BR26" s="6" t="inlineStr">
         <is>
           <t>Aceptable</t>
@@ -8890,14 +8794,8 @@
       <c r="U27" s="8" t="n">
         <v>45</v>
       </c>
-      <c r="V27" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W27" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V27" s="2" t="inlineStr"/>
+      <c r="W27" s="2" t="inlineStr"/>
       <c r="X27" s="2" t="inlineStr"/>
       <c r="Y27" s="2" t="inlineStr"/>
       <c r="Z27" s="3" t="inlineStr">
@@ -9020,14 +8918,8 @@
       <c r="BO27" s="5" t="n">
         <v>0.052</v>
       </c>
-      <c r="BP27" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BQ27" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="BP27" s="2" t="inlineStr"/>
+      <c r="BQ27" s="2" t="inlineStr"/>
       <c r="BR27" s="6" t="inlineStr">
         <is>
           <t>Aceptable</t>
@@ -9184,14 +9076,8 @@
       <c r="S28" s="2" t="inlineStr"/>
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
-      <c r="V28" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W28" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V28" s="2" t="inlineStr"/>
+      <c r="W28" s="2" t="inlineStr"/>
       <c r="X28" s="2" t="inlineStr"/>
       <c r="Y28" s="2" t="inlineStr"/>
       <c r="Z28" s="3" t="inlineStr">
@@ -9502,14 +9388,8 @@
       <c r="U29" s="8" t="n">
         <v>45</v>
       </c>
-      <c r="V29" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W29" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V29" s="2" t="inlineStr"/>
+      <c r="W29" s="2" t="inlineStr"/>
       <c r="X29" s="2" t="inlineStr"/>
       <c r="Y29" s="2" t="inlineStr"/>
       <c r="Z29" s="3" t="inlineStr">
@@ -9820,14 +9700,8 @@
       <c r="U30" s="8" t="n">
         <v>45</v>
       </c>
-      <c r="V30" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W30" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V30" s="2" t="inlineStr"/>
+      <c r="W30" s="2" t="inlineStr"/>
       <c r="X30" s="2" t="inlineStr"/>
       <c r="Y30" s="2" t="inlineStr"/>
       <c r="Z30" s="3" t="inlineStr">
@@ -10138,14 +10012,8 @@
       <c r="U31" s="8" t="n">
         <v>59</v>
       </c>
-      <c r="V31" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W31" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V31" s="2" t="inlineStr"/>
+      <c r="W31" s="2" t="inlineStr"/>
       <c r="X31" s="2" t="inlineStr"/>
       <c r="Y31" s="2" t="inlineStr"/>
       <c r="Z31" s="3" t="inlineStr">
@@ -10456,14 +10324,8 @@
       <c r="U32" s="8" t="n">
         <v>44</v>
       </c>
-      <c r="V32" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W32" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V32" s="2" t="inlineStr"/>
+      <c r="W32" s="2" t="inlineStr"/>
       <c r="X32" s="2" t="inlineStr"/>
       <c r="Y32" s="2" t="inlineStr"/>
       <c r="Z32" s="3" t="inlineStr">
@@ -10774,14 +10636,8 @@
       <c r="U33" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="V33" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W33" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V33" s="2" t="inlineStr"/>
+      <c r="W33" s="2" t="inlineStr"/>
       <c r="X33" s="2" t="inlineStr"/>
       <c r="Y33" s="2" t="inlineStr"/>
       <c r="Z33" s="3" t="inlineStr">
@@ -11092,14 +10948,8 @@
       <c r="U34" s="8" t="n">
         <v>44</v>
       </c>
-      <c r="V34" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W34" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V34" s="2" t="inlineStr"/>
+      <c r="W34" s="2" t="inlineStr"/>
       <c r="X34" s="2" t="inlineStr"/>
       <c r="Y34" s="2" t="inlineStr"/>
       <c r="Z34" s="3" t="inlineStr">
@@ -11410,14 +11260,8 @@
       <c r="U35" s="8" t="n">
         <v>42</v>
       </c>
-      <c r="V35" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W35" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V35" s="2" t="inlineStr"/>
+      <c r="W35" s="2" t="inlineStr"/>
       <c r="X35" s="2" t="inlineStr"/>
       <c r="Y35" s="2" t="inlineStr"/>
       <c r="Z35" s="3" t="inlineStr">
@@ -11728,14 +11572,8 @@
       <c r="U36" s="8" t="n">
         <v>54</v>
       </c>
-      <c r="V36" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W36" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V36" s="2" t="inlineStr"/>
+      <c r="W36" s="2" t="inlineStr"/>
       <c r="X36" s="2" t="inlineStr"/>
       <c r="Y36" s="2" t="inlineStr"/>
       <c r="Z36" s="3" t="inlineStr">
@@ -12034,14 +11872,8 @@
       <c r="U37" s="8" t="n">
         <v>46</v>
       </c>
-      <c r="V37" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W37" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V37" s="2" t="inlineStr"/>
+      <c r="W37" s="2" t="inlineStr"/>
       <c r="X37" s="2" t="inlineStr"/>
       <c r="Y37" s="2" t="inlineStr"/>
       <c r="Z37" s="3" t="inlineStr">
@@ -12352,14 +12184,8 @@
       <c r="U38" s="8" t="n">
         <v>52</v>
       </c>
-      <c r="V38" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W38" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V38" s="2" t="inlineStr"/>
+      <c r="W38" s="2" t="inlineStr"/>
       <c r="X38" s="2" t="inlineStr"/>
       <c r="Y38" s="2" t="inlineStr"/>
       <c r="Z38" s="3" t="inlineStr">
@@ -12670,14 +12496,8 @@
       <c r="U39" s="8" t="n">
         <v>46</v>
       </c>
-      <c r="V39" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W39" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V39" s="2" t="inlineStr"/>
+      <c r="W39" s="2" t="inlineStr"/>
       <c r="X39" s="2" t="inlineStr"/>
       <c r="Y39" s="2" t="inlineStr"/>
       <c r="Z39" s="3" t="inlineStr">
@@ -12994,14 +12814,8 @@
       <c r="U40" s="8" t="n">
         <v>56</v>
       </c>
-      <c r="V40" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W40" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V40" s="2" t="inlineStr"/>
+      <c r="W40" s="2" t="inlineStr"/>
       <c r="X40" s="2" t="inlineStr"/>
       <c r="Y40" s="2" t="inlineStr"/>
       <c r="Z40" s="3" t="inlineStr">
@@ -13318,14 +13132,8 @@
       <c r="U41" s="8" t="n">
         <v>46</v>
       </c>
-      <c r="V41" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W41" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V41" s="2" t="inlineStr"/>
+      <c r="W41" s="2" t="inlineStr"/>
       <c r="X41" s="2" t="inlineStr"/>
       <c r="Y41" s="2" t="inlineStr"/>
       <c r="Z41" s="3" t="inlineStr">
@@ -13518,14 +13326,8 @@
       <c r="CE41" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="CF41" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="CG41" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="CF41" s="2" t="inlineStr"/>
+      <c r="CG41" s="2" t="inlineStr"/>
       <c r="CH41" s="3" t="inlineStr">
         <is>
           <t>Buena</t>
@@ -13642,14 +13444,8 @@
       <c r="U42" s="8" t="n">
         <v>49</v>
       </c>
-      <c r="V42" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W42" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V42" s="2" t="inlineStr"/>
+      <c r="W42" s="2" t="inlineStr"/>
       <c r="X42" s="2" t="inlineStr"/>
       <c r="Y42" s="2" t="inlineStr"/>
       <c r="Z42" s="2" t="inlineStr"/>
@@ -13948,14 +13744,8 @@
       <c r="U43" s="8" t="n">
         <v>61</v>
       </c>
-      <c r="V43" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W43" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V43" s="2" t="inlineStr"/>
+      <c r="W43" s="2" t="inlineStr"/>
       <c r="X43" s="2" t="inlineStr"/>
       <c r="Y43" s="2" t="inlineStr"/>
       <c r="Z43" s="3" t="inlineStr">
@@ -14272,14 +14062,8 @@
       <c r="U44" s="8" t="n">
         <v>62</v>
       </c>
-      <c r="V44" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W44" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V44" s="2" t="inlineStr"/>
+      <c r="W44" s="2" t="inlineStr"/>
       <c r="X44" s="2" t="inlineStr"/>
       <c r="Y44" s="2" t="inlineStr"/>
       <c r="Z44" s="3" t="inlineStr">
@@ -14590,14 +14374,8 @@
       <c r="U45" s="8" t="n">
         <v>61</v>
       </c>
-      <c r="V45" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W45" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V45" s="2" t="inlineStr"/>
+      <c r="W45" s="2" t="inlineStr"/>
       <c r="X45" s="2" t="inlineStr"/>
       <c r="Y45" s="2" t="inlineStr"/>
       <c r="Z45" s="3" t="inlineStr">
@@ -14908,14 +14686,8 @@
       <c r="U46" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="V46" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W46" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V46" s="2" t="inlineStr"/>
+      <c r="W46" s="2" t="inlineStr"/>
       <c r="X46" s="2" t="inlineStr"/>
       <c r="Y46" s="2" t="inlineStr"/>
       <c r="Z46" s="3" t="inlineStr">
@@ -15226,14 +14998,8 @@
       <c r="U47" s="8" t="n">
         <v>71</v>
       </c>
-      <c r="V47" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W47" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V47" s="2" t="inlineStr"/>
+      <c r="W47" s="2" t="inlineStr"/>
       <c r="X47" s="2" t="inlineStr"/>
       <c r="Y47" s="2" t="inlineStr"/>
       <c r="Z47" s="2" t="inlineStr"/>
@@ -15526,14 +15292,8 @@
       <c r="U48" s="8" t="n">
         <v>61</v>
       </c>
-      <c r="V48" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W48" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V48" s="2" t="inlineStr"/>
+      <c r="W48" s="2" t="inlineStr"/>
       <c r="X48" s="2" t="inlineStr"/>
       <c r="Y48" s="2" t="inlineStr"/>
       <c r="Z48" s="3" t="inlineStr">
@@ -15832,14 +15592,8 @@
       <c r="U49" s="8" t="n">
         <v>66</v>
       </c>
-      <c r="V49" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W49" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V49" s="2" t="inlineStr"/>
+      <c r="W49" s="2" t="inlineStr"/>
       <c r="X49" s="2" t="inlineStr"/>
       <c r="Y49" s="2" t="inlineStr"/>
       <c r="Z49" s="3" t="inlineStr">
@@ -16138,14 +15892,8 @@
       <c r="U50" s="8" t="n">
         <v>58</v>
       </c>
-      <c r="V50" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W50" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V50" s="2" t="inlineStr"/>
+      <c r="W50" s="2" t="inlineStr"/>
       <c r="X50" s="2" t="inlineStr"/>
       <c r="Y50" s="2" t="inlineStr"/>
       <c r="Z50" s="2" t="inlineStr"/>
@@ -16444,14 +16192,8 @@
       <c r="U51" s="8" t="n">
         <v>59</v>
       </c>
-      <c r="V51" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W51" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V51" s="2" t="inlineStr"/>
+      <c r="W51" s="2" t="inlineStr"/>
       <c r="X51" s="2" t="inlineStr"/>
       <c r="Y51" s="2" t="inlineStr"/>
       <c r="Z51" s="2" t="inlineStr"/>
@@ -16756,14 +16498,8 @@
       <c r="U52" s="8" t="n">
         <v>63</v>
       </c>
-      <c r="V52" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W52" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V52" s="2" t="inlineStr"/>
+      <c r="W52" s="2" t="inlineStr"/>
       <c r="X52" s="2" t="inlineStr"/>
       <c r="Y52" s="2" t="inlineStr"/>
       <c r="Z52" s="2" t="inlineStr"/>
@@ -17044,14 +16780,8 @@
       <c r="U53" s="8" t="n">
         <v>75</v>
       </c>
-      <c r="V53" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W53" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V53" s="2" t="inlineStr"/>
+      <c r="W53" s="2" t="inlineStr"/>
       <c r="X53" s="2" t="inlineStr"/>
       <c r="Y53" s="2" t="inlineStr"/>
       <c r="Z53" s="2" t="inlineStr"/>
@@ -17308,14 +17038,8 @@
       <c r="U54" s="8" t="n">
         <v>76</v>
       </c>
-      <c r="V54" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W54" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V54" s="2" t="inlineStr"/>
+      <c r="W54" s="2" t="inlineStr"/>
       <c r="X54" s="2" t="inlineStr"/>
       <c r="Y54" s="2" t="inlineStr"/>
       <c r="Z54" s="2" t="inlineStr"/>
@@ -17566,14 +17290,8 @@
       <c r="S55" s="2" t="inlineStr"/>
       <c r="T55" s="2" t="inlineStr"/>
       <c r="U55" s="2" t="inlineStr"/>
-      <c r="V55" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W55" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V55" s="2" t="inlineStr"/>
+      <c r="W55" s="2" t="inlineStr"/>
       <c r="X55" s="2" t="inlineStr"/>
       <c r="Y55" s="2" t="inlineStr"/>
       <c r="Z55" s="2" t="inlineStr"/>
@@ -17812,14 +17530,8 @@
       <c r="S56" s="2" t="inlineStr"/>
       <c r="T56" s="2" t="inlineStr"/>
       <c r="U56" s="2" t="inlineStr"/>
-      <c r="V56" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W56" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V56" s="2" t="inlineStr"/>
+      <c r="W56" s="2" t="inlineStr"/>
       <c r="X56" s="2" t="inlineStr"/>
       <c r="Y56" s="2" t="inlineStr"/>
       <c r="Z56" s="2" t="inlineStr"/>
@@ -18070,14 +17782,8 @@
       <c r="U57" s="8" t="n">
         <v>57</v>
       </c>
-      <c r="V57" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W57" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V57" s="2" t="inlineStr"/>
+      <c r="W57" s="2" t="inlineStr"/>
       <c r="X57" s="2" t="inlineStr"/>
       <c r="Y57" s="2" t="inlineStr"/>
       <c r="Z57" s="2" t="inlineStr"/>
@@ -18352,14 +18058,8 @@
       <c r="U58" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="V58" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W58" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V58" s="2" t="inlineStr"/>
+      <c r="W58" s="2" t="inlineStr"/>
       <c r="X58" s="2" t="inlineStr"/>
       <c r="Y58" s="2" t="inlineStr"/>
       <c r="Z58" s="3" t="inlineStr">
@@ -18640,14 +18340,8 @@
       <c r="U59" s="8" t="n">
         <v>66</v>
       </c>
-      <c r="V59" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W59" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V59" s="2" t="inlineStr"/>
+      <c r="W59" s="2" t="inlineStr"/>
       <c r="X59" s="2" t="inlineStr"/>
       <c r="Y59" s="2" t="inlineStr"/>
       <c r="Z59" s="3" t="inlineStr">
@@ -18928,14 +18622,8 @@
       <c r="U60" s="8" t="n">
         <v>48</v>
       </c>
-      <c r="V60" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W60" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V60" s="2" t="inlineStr"/>
+      <c r="W60" s="2" t="inlineStr"/>
       <c r="X60" s="2" t="inlineStr"/>
       <c r="Y60" s="2" t="inlineStr"/>
       <c r="Z60" s="3" t="inlineStr">
@@ -19222,14 +18910,8 @@
       <c r="U61" s="8" t="n">
         <v>51</v>
       </c>
-      <c r="V61" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W61" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V61" s="2" t="inlineStr"/>
+      <c r="W61" s="2" t="inlineStr"/>
       <c r="X61" s="2" t="inlineStr"/>
       <c r="Y61" s="2" t="inlineStr"/>
       <c r="Z61" s="3" t="inlineStr">
@@ -19516,14 +19198,8 @@
       <c r="U62" s="8" t="n">
         <v>53</v>
       </c>
-      <c r="V62" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W62" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V62" s="2" t="inlineStr"/>
+      <c r="W62" s="2" t="inlineStr"/>
       <c r="X62" s="2" t="inlineStr"/>
       <c r="Y62" s="2" t="inlineStr"/>
       <c r="Z62" s="3" t="inlineStr">
@@ -19804,14 +19480,8 @@
       <c r="U63" s="8" t="n">
         <v>56</v>
       </c>
-      <c r="V63" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W63" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V63" s="2" t="inlineStr"/>
+      <c r="W63" s="2" t="inlineStr"/>
       <c r="X63" s="2" t="inlineStr"/>
       <c r="Y63" s="2" t="inlineStr"/>
       <c r="Z63" s="3" t="inlineStr">
@@ -20092,14 +19762,8 @@
       <c r="U64" s="8" t="n">
         <v>48</v>
       </c>
-      <c r="V64" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W64" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V64" s="2" t="inlineStr"/>
+      <c r="W64" s="2" t="inlineStr"/>
       <c r="X64" s="2" t="inlineStr"/>
       <c r="Y64" s="2" t="inlineStr"/>
       <c r="Z64" s="3" t="inlineStr">
@@ -20392,14 +20056,8 @@
       <c r="U65" s="8" t="n">
         <v>51</v>
       </c>
-      <c r="V65" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W65" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V65" s="2" t="inlineStr"/>
+      <c r="W65" s="2" t="inlineStr"/>
       <c r="X65" s="2" t="inlineStr"/>
       <c r="Y65" s="2" t="inlineStr"/>
       <c r="Z65" s="3" t="inlineStr">
@@ -20680,14 +20338,8 @@
       <c r="U66" s="8" t="n">
         <v>39</v>
       </c>
-      <c r="V66" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W66" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V66" s="2" t="inlineStr"/>
+      <c r="W66" s="2" t="inlineStr"/>
       <c r="X66" s="2" t="inlineStr"/>
       <c r="Y66" s="2" t="inlineStr"/>
       <c r="Z66" s="3" t="inlineStr">
@@ -20968,14 +20620,8 @@
       <c r="U67" s="8" t="n">
         <v>46</v>
       </c>
-      <c r="V67" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W67" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V67" s="2" t="inlineStr"/>
+      <c r="W67" s="2" t="inlineStr"/>
       <c r="X67" s="2" t="inlineStr"/>
       <c r="Y67" s="2" t="inlineStr"/>
       <c r="Z67" s="3" t="inlineStr">
@@ -21268,14 +20914,8 @@
       <c r="U68" s="8" t="n">
         <v>68</v>
       </c>
-      <c r="V68" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W68" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V68" s="2" t="inlineStr"/>
+      <c r="W68" s="2" t="inlineStr"/>
       <c r="X68" s="2" t="inlineStr"/>
       <c r="Y68" s="2" t="inlineStr"/>
       <c r="Z68" s="3" t="inlineStr">
@@ -29888,14 +29528,8 @@
       <c r="AU41" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="AV41" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AW41" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="AV41" s="2" t="inlineStr"/>
+      <c r="AW41" s="2" t="inlineStr"/>
       <c r="AX41" s="3" t="inlineStr">
         <is>
           <t>Buena</t>
@@ -29938,11 +29572,7 @@
       <c r="BI41" s="5" t="n">
         <v>0.002</v>
       </c>
-      <c r="BJ41" s="2" t="inlineStr">
-        <is>
-          <t>Aceptable</t>
-        </is>
-      </c>
+      <c r="BJ41" s="2" t="inlineStr"/>
     </row>
     <row r="42" ht="25" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
@@ -37200,14 +36830,8 @@
       <c r="AG15" s="2" t="inlineStr"/>
       <c r="AH15" s="2" t="inlineStr"/>
       <c r="AI15" s="2" t="inlineStr"/>
-      <c r="AJ15" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AK15" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="AJ15" s="2" t="inlineStr"/>
+      <c r="AK15" s="2" t="inlineStr"/>
       <c r="AL15" s="2" t="inlineStr"/>
     </row>
     <row r="16" ht="25" customHeight="1">
@@ -37444,14 +37068,8 @@
       <c r="AI17" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="AJ17" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AK17" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="AJ17" s="2" t="inlineStr"/>
+      <c r="AK17" s="2" t="inlineStr"/>
       <c r="AL17" s="2" t="inlineStr"/>
     </row>
     <row r="18" ht="25" customHeight="1">
@@ -37474,14 +37092,8 @@
       <c r="I18" s="8" t="n">
         <v>47</v>
       </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K18" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="3" t="inlineStr">
@@ -37596,14 +37208,8 @@
       <c r="I19" s="8" t="n">
         <v>42</v>
       </c>
-      <c r="J19" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K19" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="3" t="inlineStr">
@@ -37702,11 +37308,7 @@
       <c r="AK19" s="5" t="n">
         <v>0.002</v>
       </c>
-      <c r="AL19" s="2" t="inlineStr">
-        <is>
-          <t>Aceptable</t>
-        </is>
-      </c>
+      <c r="AL19" s="2" t="inlineStr"/>
     </row>
     <row r="20" ht="25" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -37728,14 +37330,8 @@
       <c r="I20" s="8" t="n">
         <v>39</v>
       </c>
-      <c r="J20" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K20" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="3" t="inlineStr">
@@ -37834,11 +37430,7 @@
       <c r="AK20" s="5" t="n">
         <v>0.002</v>
       </c>
-      <c r="AL20" s="2" t="inlineStr">
-        <is>
-          <t>Aceptable</t>
-        </is>
-      </c>
+      <c r="AL20" s="2" t="inlineStr"/>
     </row>
     <row r="21" ht="25" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
@@ -37860,14 +37452,8 @@
       <c r="I21" s="8" t="n">
         <v>43</v>
       </c>
-      <c r="J21" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K21" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="3" t="inlineStr">
@@ -37966,11 +37552,7 @@
       <c r="AK21" s="5" t="n">
         <v>0.002</v>
       </c>
-      <c r="AL21" s="2" t="inlineStr">
-        <is>
-          <t>Aceptable</t>
-        </is>
-      </c>
+      <c r="AL21" s="2" t="inlineStr"/>
     </row>
     <row r="22" ht="25" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -37992,14 +37574,8 @@
       <c r="I22" s="8" t="n">
         <v>40</v>
       </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K22" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="3" t="inlineStr">
@@ -38074,14 +37650,8 @@
       <c r="AE22" s="5" t="n">
         <v>0.058</v>
       </c>
-      <c r="AF22" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AG22" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="AF22" s="2" t="inlineStr"/>
+      <c r="AG22" s="2" t="inlineStr"/>
       <c r="AH22" s="6" t="inlineStr">
         <is>
           <t>Aceptable</t>
@@ -38098,11 +37668,7 @@
       <c r="AK22" s="5" t="n">
         <v>0.002</v>
       </c>
-      <c r="AL22" s="2" t="inlineStr">
-        <is>
-          <t>Aceptable</t>
-        </is>
-      </c>
+      <c r="AL22" s="2" t="inlineStr"/>
     </row>
     <row r="23" ht="25" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
@@ -38118,14 +37684,8 @@
       <c r="G23" s="2" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K23" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="3" t="inlineStr">
@@ -38200,14 +37760,8 @@
       <c r="AE23" s="5" t="n">
         <v>0.052</v>
       </c>
-      <c r="AF23" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AG23" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="AF23" s="2" t="inlineStr"/>
+      <c r="AG23" s="2" t="inlineStr"/>
       <c r="AH23" s="3" t="inlineStr">
         <is>
           <t>Buena</t>
@@ -38246,14 +37800,8 @@
       <c r="I24" s="8" t="n">
         <v>36</v>
       </c>
-      <c r="J24" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K24" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="3" t="inlineStr">
@@ -38328,14 +37876,8 @@
       <c r="AE24" s="5" t="n">
         <v>0.058</v>
       </c>
-      <c r="AF24" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AG24" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="AF24" s="2" t="inlineStr"/>
+      <c r="AG24" s="2" t="inlineStr"/>
       <c r="AH24" s="3" t="inlineStr">
         <is>
           <t>Buena</t>
@@ -38368,14 +37910,8 @@
       <c r="I25" s="8" t="n">
         <v>36</v>
       </c>
-      <c r="J25" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K25" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr"/>
       <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="3" t="inlineStr">
@@ -38450,14 +37986,8 @@
       <c r="AE25" s="5" t="n">
         <v>0.052</v>
       </c>
-      <c r="AF25" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AG25" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="AF25" s="2" t="inlineStr"/>
+      <c r="AG25" s="2" t="inlineStr"/>
       <c r="AH25" s="3" t="inlineStr">
         <is>
           <t>Buena</t>
@@ -38490,14 +38020,8 @@
       <c r="I26" s="8" t="n">
         <v>43</v>
       </c>
-      <c r="J26" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K26" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="3" t="inlineStr">
@@ -38572,14 +38096,8 @@
       <c r="AE26" s="5" t="n">
         <v>0.054</v>
       </c>
-      <c r="AF26" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AG26" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="AF26" s="2" t="inlineStr"/>
+      <c r="AG26" s="2" t="inlineStr"/>
       <c r="AH26" s="6" t="inlineStr">
         <is>
           <t>Aceptable</t>
@@ -38612,14 +38130,8 @@
       <c r="I27" s="8" t="n">
         <v>45</v>
       </c>
-      <c r="J27" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K27" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="3" t="inlineStr">
@@ -38694,14 +38206,8 @@
       <c r="AE27" s="5" t="n">
         <v>0.052</v>
       </c>
-      <c r="AF27" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AG27" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="AF27" s="2" t="inlineStr"/>
+      <c r="AG27" s="2" t="inlineStr"/>
       <c r="AH27" s="6" t="inlineStr">
         <is>
           <t>Aceptable</t>
@@ -38728,14 +38234,8 @@
       <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K28" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="3" t="inlineStr">
@@ -38856,14 +38356,8 @@
       <c r="I29" s="8" t="n">
         <v>45</v>
       </c>
-      <c r="J29" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K29" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr"/>
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="3" t="inlineStr">
@@ -38978,14 +38472,8 @@
       <c r="I30" s="8" t="n">
         <v>45</v>
       </c>
-      <c r="J30" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K30" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr"/>
       <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="3" t="inlineStr">
@@ -39100,14 +38588,8 @@
       <c r="I31" s="8" t="n">
         <v>59</v>
       </c>
-      <c r="J31" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K31" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr"/>
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="3" t="inlineStr">
@@ -39222,14 +38704,8 @@
       <c r="I32" s="8" t="n">
         <v>44</v>
       </c>
-      <c r="J32" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K32" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr"/>
       <c r="L32" s="2" t="inlineStr"/>
       <c r="M32" s="2" t="inlineStr"/>
       <c r="N32" s="3" t="inlineStr">
@@ -39344,14 +38820,8 @@
       <c r="I33" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="J33" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K33" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr"/>
       <c r="L33" s="2" t="inlineStr"/>
       <c r="M33" s="2" t="inlineStr"/>
       <c r="N33" s="3" t="inlineStr">
@@ -39466,14 +38936,8 @@
       <c r="I34" s="8" t="n">
         <v>44</v>
       </c>
-      <c r="J34" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K34" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr"/>
       <c r="L34" s="2" t="inlineStr"/>
       <c r="M34" s="2" t="inlineStr"/>
       <c r="N34" s="3" t="inlineStr">
@@ -39588,14 +39052,8 @@
       <c r="I35" s="8" t="n">
         <v>42</v>
       </c>
-      <c r="J35" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K35" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr"/>
       <c r="L35" s="2" t="inlineStr"/>
       <c r="M35" s="2" t="inlineStr"/>
       <c r="N35" s="3" t="inlineStr">
@@ -39710,14 +39168,8 @@
       <c r="I36" s="8" t="n">
         <v>54</v>
       </c>
-      <c r="J36" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K36" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr"/>
       <c r="L36" s="2" t="inlineStr"/>
       <c r="M36" s="2" t="inlineStr"/>
       <c r="N36" s="3" t="inlineStr">
@@ -39832,14 +39284,8 @@
       <c r="I37" s="8" t="n">
         <v>46</v>
       </c>
-      <c r="J37" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K37" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr"/>
       <c r="L37" s="2" t="inlineStr"/>
       <c r="M37" s="2" t="inlineStr"/>
       <c r="N37" s="3" t="inlineStr">
@@ -39954,14 +39400,8 @@
       <c r="I38" s="8" t="n">
         <v>52</v>
       </c>
-      <c r="J38" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K38" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr"/>
       <c r="L38" s="2" t="inlineStr"/>
       <c r="M38" s="2" t="inlineStr"/>
       <c r="N38" s="3" t="inlineStr">
@@ -40060,11 +39500,7 @@
       <c r="AK38" s="5" t="n">
         <v>0.015</v>
       </c>
-      <c r="AL38" s="2" t="inlineStr">
-        <is>
-          <t>Mala</t>
-        </is>
-      </c>
+      <c r="AL38" s="2" t="inlineStr"/>
     </row>
     <row r="39" ht="25" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
@@ -40086,14 +39522,8 @@
       <c r="I39" s="8" t="n">
         <v>46</v>
       </c>
-      <c r="J39" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K39" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J39" s="2" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr"/>
       <c r="L39" s="2" t="inlineStr"/>
       <c r="M39" s="2" t="inlineStr"/>
       <c r="N39" s="3" t="inlineStr">
@@ -40208,14 +39638,8 @@
       <c r="I40" s="8" t="n">
         <v>56</v>
       </c>
-      <c r="J40" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K40" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr"/>
       <c r="L40" s="2" t="inlineStr"/>
       <c r="M40" s="2" t="inlineStr"/>
       <c r="N40" s="3" t="inlineStr">
@@ -40330,14 +39754,8 @@
       <c r="I41" s="8" t="n">
         <v>46</v>
       </c>
-      <c r="J41" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K41" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr"/>
       <c r="L41" s="2" t="inlineStr"/>
       <c r="M41" s="2" t="inlineStr"/>
       <c r="N41" s="3" t="inlineStr">
@@ -40452,14 +39870,8 @@
       <c r="I42" s="8" t="n">
         <v>49</v>
       </c>
-      <c r="J42" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K42" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr"/>
       <c r="L42" s="2" t="inlineStr"/>
       <c r="M42" s="2" t="inlineStr"/>
       <c r="N42" s="3" t="inlineStr">
@@ -40574,14 +39986,8 @@
       <c r="I43" s="8" t="n">
         <v>61</v>
       </c>
-      <c r="J43" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K43" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J43" s="2" t="inlineStr"/>
+      <c r="K43" s="2" t="inlineStr"/>
       <c r="L43" s="2" t="inlineStr"/>
       <c r="M43" s="2" t="inlineStr"/>
       <c r="N43" s="3" t="inlineStr">
@@ -40696,14 +40102,8 @@
       <c r="I44" s="8" t="n">
         <v>62</v>
       </c>
-      <c r="J44" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K44" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J44" s="2" t="inlineStr"/>
+      <c r="K44" s="2" t="inlineStr"/>
       <c r="L44" s="2" t="inlineStr"/>
       <c r="M44" s="2" t="inlineStr"/>
       <c r="N44" s="3" t="inlineStr">
@@ -40818,14 +40218,8 @@
       <c r="I45" s="8" t="n">
         <v>61</v>
       </c>
-      <c r="J45" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K45" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J45" s="2" t="inlineStr"/>
+      <c r="K45" s="2" t="inlineStr"/>
       <c r="L45" s="2" t="inlineStr"/>
       <c r="M45" s="2" t="inlineStr"/>
       <c r="N45" s="3" t="inlineStr">
@@ -40940,14 +40334,8 @@
       <c r="I46" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="J46" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K46" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J46" s="2" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr"/>
       <c r="L46" s="2" t="inlineStr"/>
       <c r="M46" s="2" t="inlineStr"/>
       <c r="N46" s="3" t="inlineStr">
@@ -41062,14 +40450,8 @@
       <c r="I47" s="8" t="n">
         <v>71</v>
       </c>
-      <c r="J47" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K47" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J47" s="2" t="inlineStr"/>
+      <c r="K47" s="2" t="inlineStr"/>
       <c r="L47" s="2" t="inlineStr"/>
       <c r="M47" s="2" t="inlineStr"/>
       <c r="N47" s="3" t="inlineStr">
@@ -41184,14 +40566,8 @@
       <c r="I48" s="8" t="n">
         <v>61</v>
       </c>
-      <c r="J48" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K48" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J48" s="2" t="inlineStr"/>
+      <c r="K48" s="2" t="inlineStr"/>
       <c r="L48" s="2" t="inlineStr"/>
       <c r="M48" s="2" t="inlineStr"/>
       <c r="N48" s="3" t="inlineStr">
@@ -41294,14 +40670,8 @@
       <c r="I49" s="8" t="n">
         <v>66</v>
       </c>
-      <c r="J49" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K49" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J49" s="2" t="inlineStr"/>
+      <c r="K49" s="2" t="inlineStr"/>
       <c r="L49" s="2" t="inlineStr"/>
       <c r="M49" s="2" t="inlineStr"/>
       <c r="N49" s="3" t="inlineStr">
@@ -41416,14 +40786,8 @@
       <c r="I50" s="8" t="n">
         <v>58</v>
       </c>
-      <c r="J50" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K50" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J50" s="2" t="inlineStr"/>
+      <c r="K50" s="2" t="inlineStr"/>
       <c r="L50" s="2" t="inlineStr"/>
       <c r="M50" s="2" t="inlineStr"/>
       <c r="N50" s="3" t="inlineStr">
@@ -41538,14 +40902,8 @@
       <c r="I51" s="8" t="n">
         <v>59</v>
       </c>
-      <c r="J51" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K51" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J51" s="2" t="inlineStr"/>
+      <c r="K51" s="2" t="inlineStr"/>
       <c r="L51" s="2" t="inlineStr"/>
       <c r="M51" s="2" t="inlineStr"/>
       <c r="N51" s="3" t="inlineStr">
@@ -41660,14 +41018,8 @@
       <c r="I52" s="8" t="n">
         <v>63</v>
       </c>
-      <c r="J52" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K52" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J52" s="2" t="inlineStr"/>
+      <c r="K52" s="2" t="inlineStr"/>
       <c r="L52" s="2" t="inlineStr"/>
       <c r="M52" s="2" t="inlineStr"/>
       <c r="N52" s="3" t="inlineStr">
@@ -41782,14 +41134,8 @@
       <c r="I53" s="8" t="n">
         <v>75</v>
       </c>
-      <c r="J53" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K53" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J53" s="2" t="inlineStr"/>
+      <c r="K53" s="2" t="inlineStr"/>
       <c r="L53" s="2" t="inlineStr"/>
       <c r="M53" s="2" t="inlineStr"/>
       <c r="N53" s="2" t="inlineStr"/>
@@ -41880,14 +41226,8 @@
       <c r="I54" s="8" t="n">
         <v>76</v>
       </c>
-      <c r="J54" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K54" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="inlineStr"/>
       <c r="L54" s="2" t="inlineStr"/>
       <c r="M54" s="2" t="inlineStr"/>
       <c r="N54" s="2" t="inlineStr"/>
@@ -41972,14 +41312,8 @@
       <c r="G55" s="2" t="inlineStr"/>
       <c r="H55" s="2" t="inlineStr"/>
       <c r="I55" s="2" t="inlineStr"/>
-      <c r="J55" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K55" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J55" s="2" t="inlineStr"/>
+      <c r="K55" s="2" t="inlineStr"/>
       <c r="L55" s="2" t="inlineStr"/>
       <c r="M55" s="2" t="inlineStr"/>
       <c r="N55" s="2" t="inlineStr"/>
@@ -42052,14 +41386,8 @@
       <c r="G56" s="2" t="inlineStr"/>
       <c r="H56" s="2" t="inlineStr"/>
       <c r="I56" s="2" t="inlineStr"/>
-      <c r="J56" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K56" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr"/>
       <c r="L56" s="2" t="inlineStr"/>
       <c r="M56" s="2" t="inlineStr"/>
       <c r="N56" s="2" t="inlineStr"/>
@@ -42144,14 +41472,8 @@
       <c r="I57" s="8" t="n">
         <v>57</v>
       </c>
-      <c r="J57" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K57" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J57" s="2" t="inlineStr"/>
+      <c r="K57" s="2" t="inlineStr"/>
       <c r="L57" s="2" t="inlineStr"/>
       <c r="M57" s="2" t="inlineStr"/>
       <c r="N57" s="2" t="inlineStr"/>
@@ -42242,14 +41564,8 @@
       <c r="I58" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="J58" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K58" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J58" s="2" t="inlineStr"/>
+      <c r="K58" s="2" t="inlineStr"/>
       <c r="L58" s="2" t="inlineStr"/>
       <c r="M58" s="2" t="inlineStr"/>
       <c r="N58" s="2" t="inlineStr"/>
@@ -42340,14 +41656,8 @@
       <c r="I59" s="8" t="n">
         <v>66</v>
       </c>
-      <c r="J59" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K59" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J59" s="2" t="inlineStr"/>
+      <c r="K59" s="2" t="inlineStr"/>
       <c r="L59" s="2" t="inlineStr"/>
       <c r="M59" s="2" t="inlineStr"/>
       <c r="N59" s="2" t="inlineStr"/>
@@ -42438,14 +41748,8 @@
       <c r="I60" s="8" t="n">
         <v>48</v>
       </c>
-      <c r="J60" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K60" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J60" s="2" t="inlineStr"/>
+      <c r="K60" s="2" t="inlineStr"/>
       <c r="L60" s="2" t="inlineStr"/>
       <c r="M60" s="2" t="inlineStr"/>
       <c r="N60" s="2" t="inlineStr"/>
@@ -42530,14 +41834,8 @@
       <c r="I61" s="8" t="n">
         <v>51</v>
       </c>
-      <c r="J61" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K61" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr"/>
       <c r="L61" s="2" t="inlineStr"/>
       <c r="M61" s="2" t="inlineStr"/>
       <c r="N61" s="2" t="inlineStr"/>
@@ -42622,14 +41920,8 @@
       <c r="I62" s="8" t="n">
         <v>53</v>
       </c>
-      <c r="J62" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K62" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr"/>
       <c r="L62" s="2" t="inlineStr"/>
       <c r="M62" s="2" t="inlineStr"/>
       <c r="N62" s="2" t="inlineStr"/>
@@ -42708,14 +42000,8 @@
       <c r="I63" s="8" t="n">
         <v>56</v>
       </c>
-      <c r="J63" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K63" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J63" s="2" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr"/>
       <c r="L63" s="2" t="inlineStr"/>
       <c r="M63" s="2" t="inlineStr"/>
       <c r="N63" s="3" t="inlineStr">
@@ -42794,14 +42080,8 @@
       <c r="I64" s="8" t="n">
         <v>48</v>
       </c>
-      <c r="J64" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K64" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J64" s="2" t="inlineStr"/>
+      <c r="K64" s="2" t="inlineStr"/>
       <c r="L64" s="2" t="inlineStr"/>
       <c r="M64" s="2" t="inlineStr"/>
       <c r="N64" s="3" t="inlineStr">
@@ -42892,14 +42172,8 @@
       <c r="I65" s="8" t="n">
         <v>51</v>
       </c>
-      <c r="J65" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K65" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J65" s="2" t="inlineStr"/>
+      <c r="K65" s="2" t="inlineStr"/>
       <c r="L65" s="2" t="inlineStr"/>
       <c r="M65" s="2" t="inlineStr"/>
       <c r="N65" s="3" t="inlineStr">
@@ -42990,14 +42264,8 @@
       <c r="I66" s="8" t="n">
         <v>39</v>
       </c>
-      <c r="J66" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K66" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J66" s="2" t="inlineStr"/>
+      <c r="K66" s="2" t="inlineStr"/>
       <c r="L66" s="2" t="inlineStr"/>
       <c r="M66" s="2" t="inlineStr"/>
       <c r="N66" s="3" t="inlineStr">
@@ -43088,14 +42356,8 @@
       <c r="I67" s="8" t="n">
         <v>46</v>
       </c>
-      <c r="J67" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K67" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J67" s="2" t="inlineStr"/>
+      <c r="K67" s="2" t="inlineStr"/>
       <c r="L67" s="2" t="inlineStr"/>
       <c r="M67" s="2" t="inlineStr"/>
       <c r="N67" s="3" t="inlineStr">
@@ -43186,14 +42448,8 @@
       <c r="I68" s="8" t="n">
         <v>68</v>
       </c>
-      <c r="J68" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K68" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J68" s="2" t="inlineStr"/>
+      <c r="K68" s="2" t="inlineStr"/>
       <c r="L68" s="2" t="inlineStr"/>
       <c r="M68" s="2" t="inlineStr"/>
       <c r="N68" s="3" t="inlineStr">
@@ -48018,14 +47274,8 @@
       <c r="I18" s="8" t="n">
         <v>47</v>
       </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K18" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="inlineStr"/>
@@ -48050,14 +47300,8 @@
       <c r="I19" s="8" t="n">
         <v>42</v>
       </c>
-      <c r="J19" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K19" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="inlineStr"/>
@@ -48082,14 +47326,8 @@
       <c r="I20" s="8" t="n">
         <v>39</v>
       </c>
-      <c r="J20" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K20" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="inlineStr"/>
@@ -48114,14 +47352,8 @@
       <c r="I21" s="8" t="n">
         <v>43</v>
       </c>
-      <c r="J21" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K21" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="inlineStr"/>
@@ -48146,14 +47378,8 @@
       <c r="I22" s="8" t="n">
         <v>40</v>
       </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K22" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="inlineStr"/>
@@ -48172,14 +47398,8 @@
       <c r="G23" s="2" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K23" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="inlineStr"/>
@@ -48204,14 +47424,8 @@
       <c r="I24" s="8" t="n">
         <v>36</v>
       </c>
-      <c r="J24" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K24" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="inlineStr"/>
@@ -48236,14 +47450,8 @@
       <c r="I25" s="8" t="n">
         <v>36</v>
       </c>
-      <c r="J25" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K25" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr"/>
       <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="inlineStr"/>
@@ -48268,14 +47476,8 @@
       <c r="I26" s="8" t="n">
         <v>43</v>
       </c>
-      <c r="J26" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K26" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="inlineStr"/>
@@ -48300,14 +47502,8 @@
       <c r="I27" s="8" t="n">
         <v>45</v>
       </c>
-      <c r="J27" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K27" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="inlineStr"/>
@@ -48326,14 +47522,8 @@
       <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K28" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="inlineStr"/>
@@ -48358,14 +47548,8 @@
       <c r="I29" s="8" t="n">
         <v>45</v>
       </c>
-      <c r="J29" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K29" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr"/>
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="inlineStr"/>
@@ -48390,14 +47574,8 @@
       <c r="I30" s="8" t="n">
         <v>45</v>
       </c>
-      <c r="J30" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K30" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr"/>
       <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="inlineStr"/>
@@ -48422,14 +47600,8 @@
       <c r="I31" s="8" t="n">
         <v>59</v>
       </c>
-      <c r="J31" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K31" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr"/>
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="inlineStr"/>
@@ -48454,14 +47626,8 @@
       <c r="I32" s="8" t="n">
         <v>44</v>
       </c>
-      <c r="J32" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K32" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr"/>
       <c r="L32" s="2" t="inlineStr"/>
       <c r="M32" s="2" t="inlineStr"/>
       <c r="N32" s="2" t="inlineStr"/>
@@ -48486,14 +47652,8 @@
       <c r="I33" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="J33" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K33" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr"/>
       <c r="L33" s="2" t="inlineStr"/>
       <c r="M33" s="2" t="inlineStr"/>
       <c r="N33" s="2" t="inlineStr"/>
@@ -48518,14 +47678,8 @@
       <c r="I34" s="8" t="n">
         <v>44</v>
       </c>
-      <c r="J34" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K34" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr"/>
       <c r="L34" s="2" t="inlineStr"/>
       <c r="M34" s="2" t="inlineStr"/>
       <c r="N34" s="2" t="inlineStr"/>
@@ -48550,14 +47704,8 @@
       <c r="I35" s="8" t="n">
         <v>42</v>
       </c>
-      <c r="J35" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K35" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr"/>
       <c r="L35" s="2" t="inlineStr"/>
       <c r="M35" s="2" t="inlineStr"/>
       <c r="N35" s="2" t="inlineStr"/>
@@ -48582,14 +47730,8 @@
       <c r="I36" s="8" t="n">
         <v>54</v>
       </c>
-      <c r="J36" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K36" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr"/>
       <c r="L36" s="2" t="inlineStr"/>
       <c r="M36" s="2" t="inlineStr"/>
       <c r="N36" s="2" t="inlineStr"/>
@@ -48614,14 +47756,8 @@
       <c r="I37" s="8" t="n">
         <v>46</v>
       </c>
-      <c r="J37" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K37" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr"/>
       <c r="L37" s="2" t="inlineStr"/>
       <c r="M37" s="2" t="inlineStr"/>
       <c r="N37" s="2" t="inlineStr"/>
@@ -48646,14 +47782,8 @@
       <c r="I38" s="8" t="n">
         <v>52</v>
       </c>
-      <c r="J38" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K38" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr"/>
       <c r="L38" s="2" t="inlineStr"/>
       <c r="M38" s="2" t="inlineStr"/>
       <c r="N38" s="2" t="inlineStr"/>
@@ -48678,14 +47808,8 @@
       <c r="I39" s="8" t="n">
         <v>46</v>
       </c>
-      <c r="J39" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K39" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J39" s="2" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr"/>
       <c r="L39" s="2" t="inlineStr"/>
       <c r="M39" s="2" t="inlineStr"/>
       <c r="N39" s="2" t="inlineStr"/>
@@ -48710,14 +47834,8 @@
       <c r="I40" s="8" t="n">
         <v>56</v>
       </c>
-      <c r="J40" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K40" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr"/>
       <c r="L40" s="2" t="inlineStr"/>
       <c r="M40" s="2" t="inlineStr"/>
       <c r="N40" s="2" t="inlineStr"/>
@@ -48742,14 +47860,8 @@
       <c r="I41" s="8" t="n">
         <v>46</v>
       </c>
-      <c r="J41" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K41" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr"/>
       <c r="L41" s="2" t="inlineStr"/>
       <c r="M41" s="2" t="inlineStr"/>
       <c r="N41" s="2" t="inlineStr"/>
@@ -48774,14 +47886,8 @@
       <c r="I42" s="8" t="n">
         <v>49</v>
       </c>
-      <c r="J42" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K42" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr"/>
       <c r="L42" s="2" t="inlineStr"/>
       <c r="M42" s="2" t="inlineStr"/>
       <c r="N42" s="2" t="inlineStr"/>
@@ -48806,14 +47912,8 @@
       <c r="I43" s="8" t="n">
         <v>61</v>
       </c>
-      <c r="J43" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K43" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J43" s="2" t="inlineStr"/>
+      <c r="K43" s="2" t="inlineStr"/>
       <c r="L43" s="2" t="inlineStr"/>
       <c r="M43" s="2" t="inlineStr"/>
       <c r="N43" s="2" t="inlineStr"/>
@@ -48838,14 +47938,8 @@
       <c r="I44" s="8" t="n">
         <v>62</v>
       </c>
-      <c r="J44" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K44" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J44" s="2" t="inlineStr"/>
+      <c r="K44" s="2" t="inlineStr"/>
       <c r="L44" s="2" t="inlineStr"/>
       <c r="M44" s="2" t="inlineStr"/>
       <c r="N44" s="2" t="inlineStr"/>
@@ -48870,14 +47964,8 @@
       <c r="I45" s="8" t="n">
         <v>61</v>
       </c>
-      <c r="J45" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K45" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J45" s="2" t="inlineStr"/>
+      <c r="K45" s="2" t="inlineStr"/>
       <c r="L45" s="2" t="inlineStr"/>
       <c r="M45" s="2" t="inlineStr"/>
       <c r="N45" s="2" t="inlineStr"/>
@@ -48902,14 +47990,8 @@
       <c r="I46" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="J46" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K46" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J46" s="2" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr"/>
       <c r="L46" s="2" t="inlineStr"/>
       <c r="M46" s="2" t="inlineStr"/>
       <c r="N46" s="2" t="inlineStr"/>
@@ -48934,14 +48016,8 @@
       <c r="I47" s="8" t="n">
         <v>71</v>
       </c>
-      <c r="J47" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K47" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J47" s="2" t="inlineStr"/>
+      <c r="K47" s="2" t="inlineStr"/>
       <c r="L47" s="2" t="inlineStr"/>
       <c r="M47" s="2" t="inlineStr"/>
       <c r="N47" s="2" t="inlineStr"/>
@@ -48966,14 +48042,8 @@
       <c r="I48" s="8" t="n">
         <v>61</v>
       </c>
-      <c r="J48" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K48" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J48" s="2" t="inlineStr"/>
+      <c r="K48" s="2" t="inlineStr"/>
       <c r="L48" s="2" t="inlineStr"/>
       <c r="M48" s="2" t="inlineStr"/>
       <c r="N48" s="2" t="inlineStr"/>
@@ -48998,14 +48068,8 @@
       <c r="I49" s="8" t="n">
         <v>66</v>
       </c>
-      <c r="J49" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K49" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J49" s="2" t="inlineStr"/>
+      <c r="K49" s="2" t="inlineStr"/>
       <c r="L49" s="2" t="inlineStr"/>
       <c r="M49" s="2" t="inlineStr"/>
       <c r="N49" s="2" t="inlineStr"/>
@@ -49030,14 +48094,8 @@
       <c r="I50" s="8" t="n">
         <v>58</v>
       </c>
-      <c r="J50" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K50" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J50" s="2" t="inlineStr"/>
+      <c r="K50" s="2" t="inlineStr"/>
       <c r="L50" s="2" t="inlineStr"/>
       <c r="M50" s="2" t="inlineStr"/>
       <c r="N50" s="2" t="inlineStr"/>
@@ -49062,14 +48120,8 @@
       <c r="I51" s="8" t="n">
         <v>59</v>
       </c>
-      <c r="J51" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K51" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J51" s="2" t="inlineStr"/>
+      <c r="K51" s="2" t="inlineStr"/>
       <c r="L51" s="2" t="inlineStr"/>
       <c r="M51" s="2" t="inlineStr"/>
       <c r="N51" s="2" t="inlineStr"/>
@@ -49094,14 +48146,8 @@
       <c r="I52" s="8" t="n">
         <v>63</v>
       </c>
-      <c r="J52" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K52" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J52" s="2" t="inlineStr"/>
+      <c r="K52" s="2" t="inlineStr"/>
       <c r="L52" s="2" t="inlineStr"/>
       <c r="M52" s="2" t="inlineStr"/>
       <c r="N52" s="2" t="inlineStr"/>
@@ -49126,14 +48172,8 @@
       <c r="I53" s="8" t="n">
         <v>75</v>
       </c>
-      <c r="J53" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K53" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J53" s="2" t="inlineStr"/>
+      <c r="K53" s="2" t="inlineStr"/>
       <c r="L53" s="2" t="inlineStr"/>
       <c r="M53" s="2" t="inlineStr"/>
       <c r="N53" s="2" t="inlineStr"/>
@@ -49158,14 +48198,8 @@
       <c r="I54" s="8" t="n">
         <v>76</v>
       </c>
-      <c r="J54" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K54" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="inlineStr"/>
       <c r="L54" s="2" t="inlineStr"/>
       <c r="M54" s="2" t="inlineStr"/>
       <c r="N54" s="2" t="inlineStr"/>
@@ -49184,14 +48218,8 @@
       <c r="G55" s="2" t="inlineStr"/>
       <c r="H55" s="2" t="inlineStr"/>
       <c r="I55" s="2" t="inlineStr"/>
-      <c r="J55" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K55" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J55" s="2" t="inlineStr"/>
+      <c r="K55" s="2" t="inlineStr"/>
       <c r="L55" s="2" t="inlineStr"/>
       <c r="M55" s="2" t="inlineStr"/>
       <c r="N55" s="2" t="inlineStr"/>
@@ -49210,14 +48238,8 @@
       <c r="G56" s="2" t="inlineStr"/>
       <c r="H56" s="2" t="inlineStr"/>
       <c r="I56" s="2" t="inlineStr"/>
-      <c r="J56" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K56" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr"/>
       <c r="L56" s="2" t="inlineStr"/>
       <c r="M56" s="2" t="inlineStr"/>
       <c r="N56" s="2" t="inlineStr"/>
@@ -49242,14 +48264,8 @@
       <c r="I57" s="8" t="n">
         <v>57</v>
       </c>
-      <c r="J57" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K57" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J57" s="2" t="inlineStr"/>
+      <c r="K57" s="2" t="inlineStr"/>
       <c r="L57" s="2" t="inlineStr"/>
       <c r="M57" s="2" t="inlineStr"/>
       <c r="N57" s="2" t="inlineStr"/>
@@ -49274,14 +48290,8 @@
       <c r="I58" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="J58" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K58" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J58" s="2" t="inlineStr"/>
+      <c r="K58" s="2" t="inlineStr"/>
       <c r="L58" s="2" t="inlineStr"/>
       <c r="M58" s="2" t="inlineStr"/>
       <c r="N58" s="2" t="inlineStr"/>
@@ -49306,14 +48316,8 @@
       <c r="I59" s="8" t="n">
         <v>66</v>
       </c>
-      <c r="J59" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K59" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J59" s="2" t="inlineStr"/>
+      <c r="K59" s="2" t="inlineStr"/>
       <c r="L59" s="2" t="inlineStr"/>
       <c r="M59" s="2" t="inlineStr"/>
       <c r="N59" s="2" t="inlineStr"/>
@@ -49338,14 +48342,8 @@
       <c r="I60" s="8" t="n">
         <v>48</v>
       </c>
-      <c r="J60" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K60" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J60" s="2" t="inlineStr"/>
+      <c r="K60" s="2" t="inlineStr"/>
       <c r="L60" s="2" t="inlineStr"/>
       <c r="M60" s="2" t="inlineStr"/>
       <c r="N60" s="2" t="inlineStr"/>
@@ -49370,14 +48368,8 @@
       <c r="I61" s="8" t="n">
         <v>51</v>
       </c>
-      <c r="J61" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K61" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr"/>
       <c r="L61" s="2" t="inlineStr"/>
       <c r="M61" s="2" t="inlineStr"/>
       <c r="N61" s="2" t="inlineStr"/>
@@ -49402,14 +48394,8 @@
       <c r="I62" s="8" t="n">
         <v>53</v>
       </c>
-      <c r="J62" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K62" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr"/>
       <c r="L62" s="2" t="inlineStr"/>
       <c r="M62" s="2" t="inlineStr"/>
       <c r="N62" s="2" t="inlineStr"/>
@@ -49434,14 +48420,8 @@
       <c r="I63" s="8" t="n">
         <v>56</v>
       </c>
-      <c r="J63" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K63" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J63" s="2" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr"/>
       <c r="L63" s="2" t="inlineStr"/>
       <c r="M63" s="2" t="inlineStr"/>
       <c r="N63" s="2" t="inlineStr"/>
@@ -49466,14 +48446,8 @@
       <c r="I64" s="8" t="n">
         <v>48</v>
       </c>
-      <c r="J64" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K64" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J64" s="2" t="inlineStr"/>
+      <c r="K64" s="2" t="inlineStr"/>
       <c r="L64" s="2" t="inlineStr"/>
       <c r="M64" s="2" t="inlineStr"/>
       <c r="N64" s="2" t="inlineStr"/>
@@ -49498,14 +48472,8 @@
       <c r="I65" s="8" t="n">
         <v>51</v>
       </c>
-      <c r="J65" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K65" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J65" s="2" t="inlineStr"/>
+      <c r="K65" s="2" t="inlineStr"/>
       <c r="L65" s="2" t="inlineStr"/>
       <c r="M65" s="2" t="inlineStr"/>
       <c r="N65" s="2" t="inlineStr"/>
@@ -49530,14 +48498,8 @@
       <c r="I66" s="8" t="n">
         <v>39</v>
       </c>
-      <c r="J66" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K66" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J66" s="2" t="inlineStr"/>
+      <c r="K66" s="2" t="inlineStr"/>
       <c r="L66" s="2" t="inlineStr"/>
       <c r="M66" s="2" t="inlineStr"/>
       <c r="N66" s="2" t="inlineStr"/>
@@ -49562,14 +48524,8 @@
       <c r="I67" s="8" t="n">
         <v>46</v>
       </c>
-      <c r="J67" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K67" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J67" s="2" t="inlineStr"/>
+      <c r="K67" s="2" t="inlineStr"/>
       <c r="L67" s="2" t="inlineStr"/>
       <c r="M67" s="2" t="inlineStr"/>
       <c r="N67" s="2" t="inlineStr"/>
@@ -49594,14 +48550,8 @@
       <c r="I68" s="8" t="n">
         <v>68</v>
       </c>
-      <c r="J68" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K68" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J68" s="2" t="inlineStr"/>
+      <c r="K68" s="2" t="inlineStr"/>
       <c r="L68" s="2" t="inlineStr"/>
       <c r="M68" s="2" t="inlineStr"/>
       <c r="N68" s="2" t="inlineStr"/>
@@ -59360,14 +58310,8 @@
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="M15" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="inlineStr"/>
     </row>
     <row r="16" ht="25" customHeight="1">
@@ -59476,14 +58420,8 @@
       <c r="K17" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="L17" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="M17" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
       <c r="N17" s="6" t="inlineStr">
         <is>
           <t>Aceptable</t>
@@ -59754,14 +58692,8 @@
       <c r="G22" s="5" t="n">
         <v>0.058</v>
       </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="I22" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="6" t="inlineStr">
         <is>
           <t>Aceptable</t>
@@ -59814,14 +58746,8 @@
       <c r="G23" s="5" t="n">
         <v>0.052</v>
       </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="I23" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="3" t="inlineStr">
         <is>
           <t>Buena</t>
@@ -59874,14 +58800,8 @@
       <c r="G24" s="5" t="n">
         <v>0.058</v>
       </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="I24" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="3" t="inlineStr">
         <is>
           <t>Buena</t>
@@ -59892,11 +58812,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr"/>
-      <c r="N24" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
+      <c r="N24" s="2" t="inlineStr"/>
     </row>
     <row r="25" ht="25" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
@@ -59928,14 +58844,8 @@
       <c r="G25" s="5" t="n">
         <v>0.052</v>
       </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="I25" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="3" t="inlineStr">
         <is>
           <t>Buena</t>
@@ -59946,11 +58856,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr"/>
-      <c r="N25" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
+      <c r="N25" s="2" t="inlineStr"/>
     </row>
     <row r="26" ht="25" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -59982,14 +58888,8 @@
       <c r="G26" s="5" t="n">
         <v>0.054</v>
       </c>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="I26" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="6" t="inlineStr">
         <is>
           <t>Aceptable</t>
@@ -60000,11 +58900,7 @@
       </c>
       <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="inlineStr"/>
-      <c r="N26" s="6" t="inlineStr">
-        <is>
-          <t>Aceptable</t>
-        </is>
-      </c>
+      <c r="N26" s="2" t="inlineStr"/>
     </row>
     <row r="27" ht="25" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
@@ -60036,14 +58932,8 @@
       <c r="G27" s="5" t="n">
         <v>0.052</v>
       </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="I27" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="6" t="inlineStr">
         <is>
           <t>Aceptable</t>
@@ -60054,11 +58944,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="inlineStr"/>
-      <c r="N27" s="6" t="inlineStr">
-        <is>
-          <t>Aceptable</t>
-        </is>
-      </c>
+      <c r="N27" s="2" t="inlineStr"/>
     </row>
     <row r="28" ht="25" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
@@ -64528,14 +63414,8 @@
       <c r="K41" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="L41" s="3" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="M41" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="L41" s="2" t="inlineStr"/>
+      <c r="M41" s="2" t="inlineStr"/>
       <c r="N41" s="6" t="inlineStr">
         <is>
           <t>Aceptable</t>

</xml_diff>